<commit_message>
UI: aggiunto pulsante 'Roster' in sidebar; Roster: colonna 'Numero' visibile a due cifre (grid 4ch, input 3ch); piccoli aggiustamenti CSS
</commit_message>
<xml_diff>
--- a/coppa OSG 2001 All Set-1.xlsx
+++ b/coppa OSG 2001 All Set-1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\STEFANO\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\STEFANO\Desktop\My-Volley-Scout\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96765E5B-C865-49BB-A56A-2025959893B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18023695-1368-462E-ABCC-CFDEEE521829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -364,9 +364,6 @@
     <t>Dell'Acqua</t>
   </si>
   <si>
-    <t>'10</t>
-  </si>
-  <si>
     <t>GIULY</t>
   </si>
   <si>
@@ -494,6 +491,9 @@
   </si>
   <si>
     <t>Rotazione Nostra Iniziale</t>
+  </si>
+  <si>
+    <t>13</t>
   </si>
 </sst>
 </file>
@@ -529,8 +529,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -875,135 +876,135 @@
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D7" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F9" t="s">
         <v>108</v>
@@ -1011,16 +1012,16 @@
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F10" t="s">
         <v>108</v>
@@ -1028,24 +1029,24 @@
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F11" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B12" t="s">
-        <v>112</v>
+      <c r="B12" s="1" t="s">
+        <v>155</v>
       </c>
       <c r="C12" t="s">
         <v>111</v>
@@ -1234,7 +1235,7 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -1242,7 +1243,7 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.3">
@@ -1503,7 +1504,7 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -1511,7 +1512,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.3">
@@ -1762,7 +1763,7 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -1770,7 +1771,7 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.3">
@@ -1848,12 +1849,12 @@
   <sheetData>
     <row r="6" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -1871,12 +1872,12 @@
   <sheetData>
     <row r="6" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -1894,12 +1895,12 @@
   <sheetData>
     <row r="6" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix: data coerente senza timezone; split giorno/mese/anno; anteprima italiana; supporto PGS/CSI; date elenco dd/mm/yyyy
</commit_message>
<xml_diff>
--- a/coppa OSG 2001 All Set-1.xlsx
+++ b/coppa OSG 2001 All Set-1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\STEFANO\Desktop\My-Volley-Scout\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18023695-1368-462E-ABCC-CFDEEE521829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7248D9E1-DDE8-41FE-BE99-27F96D224E0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="El. Gioc." sheetId="7" r:id="rId1"/>
@@ -265,9 +265,6 @@
     <t>06r4 03a5</t>
   </si>
   <si>
-    <t>03b2 03d5 01a5</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
@@ -494,6 +491,9 @@
   </si>
   <si>
     <t>13</t>
+  </si>
+  <si>
+    <t>03b2 03d5 01a1</t>
   </si>
 </sst>
 </file>
@@ -876,348 +876,348 @@
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C7" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C12" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E12" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C13" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D13" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E13" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F14" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C15" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D15" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E15" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C16" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D16" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C20" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D20" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E20" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F20" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.3">
       <c r="C21" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D21" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.3">
       <c r="C22" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D22" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
       <c r="C23" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D23" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.3">
       <c r="C24" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D24" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1235,7 +1235,7 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -1243,7 +1243,7 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.3">
@@ -1504,7 +1504,7 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -1512,7 +1512,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.3">
@@ -1757,13 +1757,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A6:B29"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="22.09765625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -1771,7 +1774,7 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.3">
@@ -1831,13 +1834,13 @@
     </row>
     <row r="29" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B29" t="s">
-        <v>79</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:B2 A4:B5 B3 A8:B29" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:B2 A4:B5 B3 A8:B28 A29" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1849,12 +1852,12 @@
   <sheetData>
     <row r="6" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -1872,12 +1875,12 @@
   <sheetData>
     <row r="6" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -1895,12 +1898,12 @@
   <sheetData>
     <row r="6" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>